<commit_message>
feat(banner): new 2026 games lineup (Dune Awakening, CONTROL Resonant, EA FC 27, Silent Hill Townfall)
Replace the old placeholder banner slides with the four new 2026
showcase titles, updated via banner/source.xlsx and regenerated
banner/data.json (npm run banner-excel-to-json).

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/banner/source.xlsx
+++ b/banner/source.xlsx
@@ -1,41 +1,65 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bo2lz\Desktop\Drive Deals V1.0\Drive Deals V1.0\banner\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76AD47DA-6BE6-4F45-B4C1-B57BB926ED2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-16320" yWindow="-6030" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="banner" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+  <si>
+    <t>title</t>
+  </si>
+  <si>
+    <t>image</t>
+  </si>
+  <si>
+    <t>sizeGB</t>
+  </si>
+  <si>
+    <t>Dune - Awakening</t>
+  </si>
+  <si>
+    <t>Dune - Awakening.jpg</t>
+  </si>
+  <si>
+    <t>CONTROL Resonant</t>
+  </si>
+  <si>
+    <t>CONTROL Resonant.jpg</t>
+  </si>
+  <si>
+    <t>EA Sports FC 27</t>
+  </si>
+  <si>
+    <t>EA Sports FC 27.jpg</t>
+  </si>
+  <si>
+    <t>SILENT HILL - Townfall</t>
+  </si>
+  <si>
+    <t>SILENT HILL - Townfall.jpg</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -65,13 +89,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,67 +428,73 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>title</v>
-      </c>
-      <c r="B1" t="str">
-        <v>image</v>
-      </c>
-      <c r="C1" t="str">
-        <v>sizeGB</v>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>New Release 1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>game-001.jpg</v>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
       </c>
       <c r="C2">
-        <v>10.6</v>
+        <v>24.2</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>New Release 2</v>
-      </c>
-      <c r="B3" t="str">
-        <v>film-001.jpg</v>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
       </c>
       <c r="C3">
-        <v>54.9</v>
+        <v>64.25</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>New Release 3</v>
-      </c>
-      <c r="B4" t="str">
-        <v>anime-001.jpg</v>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
       </c>
       <c r="C4">
-        <v>22.4</v>
+        <v>61.1</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>New Release 4</v>
-      </c>
-      <c r="B5" t="str">
-        <v>series-001.jpg</v>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>10</v>
       </c>
       <c r="C5">
-        <v>8.3</v>
+        <v>42.9</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C5"/>
+    <ignoredError sqref="A1:C1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(data): add 4 new games and refresh the top banner lineup
- +4 library items in games: BEAM NG, End of Abyss, Gears of War - E-Day, The Witcher 3 - Remastered
- -0 library items
- banner lineup replaced 4 for 4: dropped Dune - Awakening, CONTROL Resonant, EA Sports FC 27, SILENT HILL - Townfall
- +8 new images (4 library, 4 banner), -4 old banner images
- regenerated data.json and banner/data.json from source.xlsx
- .gitignore: ignore image-edit-tmp/
</commit_message>
<xml_diff>
--- a/banner/source.xlsx
+++ b/banner/source.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bo2lz\Desktop\Drive Deals V1.0\Drive Deals V1.0\banner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76AD47DA-6BE6-4F45-B4C1-B57BB926ED2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06D95E26-327C-4B2A-B45C-178DD3F44741}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-16320" yWindow="-6030" windowWidth="16440" windowHeight="28320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="banner" sheetId="1" r:id="rId1"/>
@@ -31,28 +31,28 @@
     <t>sizeGB</t>
   </si>
   <si>
-    <t>Dune - Awakening</t>
-  </si>
-  <si>
-    <t>Dune - Awakening.jpg</t>
-  </si>
-  <si>
-    <t>CONTROL Resonant</t>
-  </si>
-  <si>
-    <t>CONTROL Resonant.jpg</t>
-  </si>
-  <si>
-    <t>EA Sports FC 27</t>
-  </si>
-  <si>
-    <t>EA Sports FC 27.jpg</t>
-  </si>
-  <si>
-    <t>SILENT HILL - Townfall</t>
-  </si>
-  <si>
-    <t>SILENT HILL - Townfall.jpg</t>
+    <t xml:space="preserve">Gears of War - E-Day </t>
+  </si>
+  <si>
+    <t>Gears of War - E-Day .jpg</t>
+  </si>
+  <si>
+    <t>End of Abyss</t>
+  </si>
+  <si>
+    <t>End of Abyss.jpg</t>
+  </si>
+  <si>
+    <t>BEAM NG</t>
+  </si>
+  <si>
+    <t>BEAM NG.jpg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The Witcher 3 - Remastered </t>
+  </si>
+  <si>
+    <t>The Witcher 3 - Remastered .jpg</t>
   </si>
 </sst>
 </file>
@@ -455,7 +455,7 @@
         <v>4</v>
       </c>
       <c r="C2">
-        <v>24.2</v>
+        <v>84.5</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -466,7 +466,7 @@
         <v>6</v>
       </c>
       <c r="C3">
-        <v>64.25</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -477,7 +477,7 @@
         <v>8</v>
       </c>
       <c r="C4">
-        <v>61.1</v>
+        <v>21.8</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -488,7 +488,7 @@
         <v>10</v>
       </c>
       <c r="C5">
-        <v>42.9</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>